<commit_message>
scan: seg6 2026-07-10 18:58 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-09.xlsx
@@ -898,21 +898,21 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6579</v>
+        <v>6782</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>研揚</t>
+          <t>視陽</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>830.0519318813801</v>
+        <v>816.4694015700398</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>168</v>
+        <v>208</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,16 +923,16 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>55.65079568800395</v>
+        <v>61.2161079898446</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>22.69065329718225</v>
+        <v>18.98883101348961</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.92462148803372</v>
+        <v>1.738489463039223</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.7628516712453965</v>
+        <v>1.851998813488339</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6782</v>
+        <v>6790</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>視陽</t>
+          <t>永豐實</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>816.4694015700398</v>
+        <v>797.5848642475654</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>208</v>
+        <v>40.6</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,16 +976,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>61.2161079898446</v>
+        <v>56.06017041130701</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>18.98883101348961</v>
+        <v>27.42534162084732</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.738489463039223</v>
+        <v>2.216894408836775</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.851998813488339</v>
+        <v>0.0200650518973029</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6672</v>
+        <v>6579</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>騰輝電子-KY</t>
+          <t>研揚</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>813.9820381707417</v>
+        <v>790.0519318813801</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>298</v>
+        <v>168</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>63.28453907555873</v>
+        <v>55.65079568800395</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>44.90669516572874</v>
+        <v>22.69065329718225</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.4074601068240206</v>
+        <v>0.92462148803372</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.909622065573938</v>
+        <v>0.7628516712453965</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1057,21 +1057,21 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6790</v>
+        <v>6672</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>永豐實</t>
+          <t>騰輝電子-KY</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>797.5848642475654</v>
+        <v>773.9820381707417</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>40.6</v>
+        <v>298</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56.06017041130701</v>
+        <v>63.28453907555873</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>27.42534162084732</v>
+        <v>44.90669516572874</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2.216894408836775</v>
+        <v>0.4074601068240206</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,11 +1100,11 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0200650518973029</v>
+        <v>0.909622065573938</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>785.1053716558544</v>
+        <v>745.1053716558544</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>199.5</v>
@@ -1852,21 +1852,21 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6526</v>
+        <v>6494</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>620.8358868881099</v>
+        <v>605.6281069906465</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>652</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,49 +1877,49 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46.55920794044477</v>
+        <v>54.75708981889597</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>12.50977640156015</v>
+        <v>30.79711053846729</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.3180578006867144</v>
+        <v>0.4960974403011379</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-3.836454092270575</v>
+        <v>-0.4436447065226803</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6494</v>
+        <v>6548</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>長科*</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>605.6281069906465</v>
+        <v>605.0684096141974</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>65.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,49 +1930,49 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>54.75708981889597</v>
+        <v>49.32164392833502</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>30.79711053846729</v>
+        <v>35.19220546615367</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.4960974403011379</v>
+        <v>0.4280797026316167</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.4436447065226803</v>
+        <v>-1.606830051550298</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6548</v>
+        <v>6776</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>長科*</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>605.0684096141974</v>
+        <v>602.1172151615042</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>82.90000000000001</v>
+        <v>55.7</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,49 +1983,49 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>49.32164392833502</v>
+        <v>44.07719400615863</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>35.19220546615367</v>
+        <v>15.16728503789413</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.4280797026316167</v>
+        <v>0.4556270969896387</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-1.606830051550298</v>
+        <v>0.007830528605297499</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6776</v>
+        <v>6719</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>力智</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>602.1172151615042</v>
+        <v>600.4071475628472</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>55.7</v>
+        <v>266.5</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>44.07719400615863</v>
+        <v>50.77748288044828</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>15.16728503789413</v>
+        <v>36.36714290865228</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.4556270969896387</v>
+        <v>0.4679120686323972</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.007830528605297499</v>
+        <v>-2.178105202121177</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6719</v>
+        <v>6534</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>力智</t>
+          <t>正瀚-創</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>600.4071475628472</v>
+        <v>596.5304830346231</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>266.5</v>
+        <v>93</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>50.77748288044828</v>
+        <v>56.377685820084</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>36.36714290865228</v>
+        <v>15.95026664477515</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.4679120686323972</v>
+        <v>1.365323079628226</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-2.178105202121177</v>
+        <v>0.3359677804920924</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6534</v>
+        <v>6651</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>正瀚-創</t>
+          <t>全宇昕</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>596.5304830346231</v>
+        <v>596.327139434096</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>93</v>
+        <v>153</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>56.377685820084</v>
+        <v>52.85462862539603</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>15.95026664477515</v>
+        <v>29.15820876787029</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.365323079628226</v>
+        <v>0.5657071327213851</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.3359677804920924</v>
+        <v>-0.3302301955753322</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6651</v>
+        <v>6693</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>全宇昕</t>
+          <t>廣閎科</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>596.327139434096</v>
+        <v>592.7668022939393</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>153</v>
+        <v>236.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>52.85462862539603</v>
+        <v>57.38882725730897</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>29.15820876787029</v>
+        <v>48.35219013904855</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.5657071327213851</v>
+        <v>0.7093456386997857</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.3302301955753322</v>
+        <v>-0.8913554387701943</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6693</v>
+        <v>6829</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>廣閎科</t>
+          <t>千附精密</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>592.7668022939393</v>
+        <v>582.0746388788924</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>236.5</v>
+        <v>222</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.38882725730897</v>
+        <v>53.37132264412852</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>48.35219013904855</v>
+        <v>12.80794466052242</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.7093456386997857</v>
+        <v>1.029161936934242</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.8913554387701943</v>
+        <v>0.134213562158755</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6829</v>
+        <v>6526</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>千附精密</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>582.0746388788924</v>
+        <v>580.8358868881099</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>222</v>
+        <v>652</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,29 +2301,29 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>53.37132264412852</v>
+        <v>46.55920794044477</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>12.80794466052242</v>
+        <v>12.50977640156015</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.029161936934242</v>
+        <v>0.3180578006867144</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M35" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.134213562158755</v>
+        <v>-3.836454092270575</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6641</v>
+        <v>6757</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>台灣虎航-創</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>541.3480499949726</v>
+        <v>539.6201191390852</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>18.55</v>
+        <v>58.2</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.15916601029208</v>
+        <v>47.89947150532576</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>21.53463700116355</v>
+        <v>33.4044542250839</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.2348049994972524</v>
+        <v>0.3874529482200982</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.0789543981768993</v>
+        <v>-0.510026576499796</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6757</v>
+        <v>6556</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>台灣虎航-創</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>539.6201191390852</v>
+        <v>537.7912947879956</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>58.2</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.89947150532576</v>
+        <v>43.50049532804022</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>33.4044542250839</v>
+        <v>25.4175389739355</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.3874529482200982</v>
+        <v>4.507926746338204</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.510026576499796</v>
+        <v>-0.193538167136914</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6556</v>
+        <v>6613</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>朋億*</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>537.7912947879956</v>
+        <v>532.2781759184518</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>70.59999999999999</v>
+        <v>321</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>43.50049532804022</v>
+        <v>48.1548853306832</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>25.4175389739355</v>
+        <v>26.18091668333613</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>4.507926746338204</v>
+        <v>0.3491639708233205</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.193538167136914</v>
+        <v>-8.294732397284093</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6668</v>
+        <v>6486</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>534.0954600328597</v>
+        <v>526.4315539908017</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>37.9</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>44.24061600837763</v>
+        <v>54.46584108495598</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>17.49634825636789</v>
+        <v>22.52926446869758</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.2315904586944201</v>
+        <v>0.7014900816502103</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.5166812948567168</v>
+        <v>0.2434784200002912</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6613</v>
+        <v>6541</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>朋億*</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>532.2781759184518</v>
+        <v>520.788563706419</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>321</v>
+        <v>40.8</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>48.1548853306832</v>
+        <v>50.37825055393518</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>26.18091668333613</v>
+        <v>15.95431463490334</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.3491639708233205</v>
+        <v>0.4791819830682827</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-8.294732397284093</v>
+        <v>-0.0515945649777843</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6669</v>
+        <v>6684</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>安格</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>527.7527193266883</v>
+        <v>513.5871514814752</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>5040</v>
+        <v>53.9</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,49 +3043,49 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>51.96524510439431</v>
+        <v>48.12188760072574</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>13.16601854784374</v>
+        <v>34.74033046096234</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.239935985599949</v>
+        <v>0.2555517275361595</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>35.82695697358312</v>
+        <v>-0.844057614690052</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6486</v>
+        <v>6722</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>互動</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>526.4315539908017</v>
+        <v>509.7704691092051</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>83.09999999999999</v>
+        <v>35.45</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>54.46584108495598</v>
+        <v>41.78422157427065</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>22.52926446869758</v>
+        <v>36.62134005229357</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.7014900816502103</v>
+        <v>0.1865728134092482</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.2434784200002912</v>
+        <v>0.0319693211539622</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6541</v>
+        <v>6771</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>520.788563706419</v>
+        <v>505.9485006770078</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>40.8</v>
+        <v>39.8</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>50.37825055393518</v>
+        <v>44.11121485010584</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>15.95431463490334</v>
+        <v>20.97283053484768</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4791819830682827</v>
+        <v>0.3808665749470042</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0515945649777843</v>
+        <v>0.0462064449937836</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6684</v>
+        <v>6641</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>安格</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>513.5871514814752</v>
+        <v>501.3480499949725</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>53.9</v>
+        <v>18.55</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>48.12188760072574</v>
+        <v>52.15916601029208</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>34.74033046096234</v>
+        <v>21.53463700116355</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.2555517275361595</v>
+        <v>0.2348049994972524</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.844057614690052</v>
+        <v>0.0789543981768993</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6722</v>
+        <v>6756</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>509.7704691092051</v>
+        <v>498.5706487819775</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>35.45</v>
+        <v>99.7</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>41.78422157427065</v>
+        <v>51.11622393290391</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>36.62134005229357</v>
+        <v>18.43002931375125</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.1865728134092482</v>
+        <v>0.719580924508797</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0319693211539622</v>
+        <v>-0.0941166256695159</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6771</v>
+        <v>6805</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>505.9485006770078</v>
+        <v>498.2261690857841</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>39.8</v>
+        <v>1460</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>44.11121485010584</v>
+        <v>35.04999473985863</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>20.97283053484768</v>
+        <v>23.31580815943655</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3808665749470042</v>
+        <v>1.466381395435663</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0462064449937836</v>
+        <v>-27.45016259752049</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6756</v>
+        <v>6530</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>498.5706487819775</v>
+        <v>496.8663280777081</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>99.7</v>
+        <v>83</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>51.11622393290391</v>
+        <v>35.42061692529114</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.43002931375125</v>
+        <v>22.55340177651775</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.719580924508797</v>
+        <v>0.6051592319693341</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.0941166256695159</v>
+        <v>-0.1612898038329095</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6805</v>
+        <v>6668</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>498.2261690857841</v>
+        <v>494.0954600328597</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>1460</v>
+        <v>37.9</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>35.04999473985863</v>
+        <v>44.24061600837763</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>23.31580815943655</v>
+        <v>17.49634825636789</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.466381395435663</v>
+        <v>0.2315904586944201</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-27.45016259752049</v>
+        <v>-0.5166812948567168</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6530</v>
+        <v>6669</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>496.8663280777081</v>
+        <v>487.7527193266883</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>83</v>
+        <v>5040</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,29 +3467,29 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>35.42061692529114</v>
+        <v>51.96524510439431</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>22.55340177651775</v>
+        <v>13.16601854784374</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.6051592319693341</v>
+        <v>1.239935985599949</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.1612898038329095</v>
+        <v>35.82695697358312</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -3548,21 +3548,21 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6581</v>
+        <v>6691</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>洋基工程</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>487.4493408512781</v>
+        <v>484.1849016766411</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>106.5</v>
+        <v>708</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>43.64214916955456</v>
+        <v>47.83081928113256</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>11.34799022438651</v>
+        <v>26.21879230494516</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1.861734772157725</v>
+        <v>0.3184901676641075</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0759752293400259</v>
+        <v>-8.401246741242378</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6691</v>
+        <v>6830</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>洋基工程</t>
+          <t>汎銓</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>484.1849016766411</v>
+        <v>482.9114658730273</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>708</v>
+        <v>416.5</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>47.83081928113256</v>
+        <v>31.57675210294522</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>26.21879230494516</v>
+        <v>25.83060349809814</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.3184901676641075</v>
+        <v>0.8696450274370079</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-8.401246741242378</v>
+        <v>-4.110552602012078</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6830</v>
+        <v>6788</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>汎銓</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>482.9114658730273</v>
+        <v>481.9701892520345</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>416.5</v>
+        <v>403.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,49 +3679,49 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>31.57675210294522</v>
+        <v>42.06927033991832</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>25.83060349809814</v>
+        <v>8.618651842756288</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.8696450274370079</v>
+        <v>0.4669477995439862</v>
       </c>
       <c r="K61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L61" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M61" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-4.110552602012078</v>
+        <v>-3.771028098114664</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6788</v>
+        <v>6614</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>481.9701892520345</v>
+        <v>472.1724104726767</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>403.5</v>
+        <v>40</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,49 +3732,49 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>42.06927033991832</v>
+        <v>49.11212072275216</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>8.618651842756288</v>
+        <v>20.77426729531906</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.4669477995439862</v>
+        <v>0.4194081595047057</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M62" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-3.771028098114664</v>
+        <v>0.0148271299643166</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6614</v>
+        <v>6581</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>472.1724104726767</v>
+        <v>467.4493408512781</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>40</v>
+        <v>106.5</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>49.11212072275216</v>
+        <v>43.64214916955456</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>20.77426729531906</v>
+        <v>11.34799022438651</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.4194081595047057</v>
+        <v>1.861734772157725</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>1</v>
@@ -3803,11 +3803,11 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0148271299643166</v>
+        <v>-0.0759752293400259</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6531</v>
+        <v>6725</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>383.7554484383441</v>
+        <v>383.5367904348528</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>922</v>
+        <v>305.5</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>44.93989250651241</v>
+        <v>43.21693973076976</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.70161541490256</v>
+        <v>21.50047520525937</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.6913528299949102</v>
+        <v>0.1970419132930303</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-13.47024695107131</v>
+        <v>-3.411320418058653</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6725</v>
+        <v>6561</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>383.5367904348528</v>
+        <v>381.3219879093637</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>305.5</v>
+        <v>330.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>43.21693973076976</v>
+        <v>39.09196338881269</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>21.50047520525937</v>
+        <v>20.63001740319667</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.1970419132930303</v>
+        <v>0.3129231034568797</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-3.411320418058653</v>
+        <v>-0.1680527533914375</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6561</v>
+        <v>6690</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>381.3219879093637</v>
+        <v>379.4332732063193</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>330.5</v>
+        <v>166.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>39.09196338881269</v>
+        <v>44.63014541075785</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>20.63001740319667</v>
+        <v>14.43662579867491</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.3129231034568797</v>
+        <v>0.3219020244547579</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.1680527533914375</v>
+        <v>-0.3006336229487034</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6690</v>
+        <v>6789</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>采鈺</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>379.4332732063193</v>
+        <v>378.5211467168094</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>166.5</v>
+        <v>515</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>44.63014541075785</v>
+        <v>49.29976006274612</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>14.43662579867491</v>
+        <v>11.45613657085052</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.3219020244547579</v>
+        <v>0.5078244177819691</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>4</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.3006336229487034</v>
+        <v>-0.7010781471795562</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6789</v>
+        <v>6597</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>采鈺</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>378.5211467168094</v>
+        <v>376.4787716480552</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>515</v>
+        <v>67.8</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>49.29976006274612</v>
+        <v>51.52220358926256</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>11.45613657085052</v>
+        <v>14.4416454967116</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.5078244177819691</v>
+        <v>0.2217467632214176</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.7010781471795562</v>
+        <v>-2.553841087692786</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6597</v>
+        <v>6715</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>376.4787716480552</v>
+        <v>375.7961387345421</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>67.8</v>
+        <v>391.5</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>51.52220358926256</v>
+        <v>41.02153305558943</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>14.4416454967116</v>
+        <v>17.16508098089622</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.2217467632214176</v>
+        <v>2.332115911198549</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-2.553841087692786</v>
+        <v>-6.670494945067979</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, williams_r_recovery</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6515</v>
+        <v>6741</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>376.1627714219665</v>
+        <v>375.1821582725876</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>7765</v>
+        <v>60</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,49 +5163,49 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>40.32504192944973</v>
+        <v>40.98150273237917</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>15.73228471199892</v>
+        <v>9.099618418777792</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.7537787896570529</v>
+        <v>1.474235345176557</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M89" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-129.3450513143999</v>
+        <v>-0.1252753070053037</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6715</v>
+        <v>6510</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>375.7961387345421</v>
+        <v>372.8793682236349</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>391.5</v>
+        <v>2855</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,49 +5216,49 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>41.02153305558943</v>
+        <v>37.5037168934422</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>17.16508098089622</v>
+        <v>20.50776648792229</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>2.332115911198549</v>
+        <v>0.6169599725795567</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M90" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-6.670494945067979</v>
+        <v>-53.90204377594968</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6741</v>
+        <v>6763</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>375.1821582725876</v>
+        <v>372.2888543904213</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>60</v>
+        <v>45.9</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>40.98150273237917</v>
+        <v>44.24551976832949</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>9.099618418777792</v>
+        <v>14.3906360408211</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.474235345176557</v>
+        <v>0.7669989018105312</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1252753070053037</v>
+        <v>-0.1506834430244326</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6510</v>
+        <v>6640</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>372.8793682236349</v>
+        <v>366.708003289398</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>2855</v>
+        <v>995</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,49 +5322,49 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.5037168934422</v>
+        <v>38.78904336163709</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>20.50776648792229</v>
+        <v>19.61234233846608</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.6169599725795567</v>
+        <v>0.6161250987838414</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M92" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-53.90204377594968</v>
+        <v>2.992810436708212</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6763</v>
+        <v>6588</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>372.2888543904213</v>
+        <v>365.7707035167654</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>45.9</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>44.24551976832949</v>
+        <v>27.44225560475532</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>14.3906360408211</v>
+        <v>21.34932604040345</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.7669989018105312</v>
+        <v>0.5217914986181071</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.1506834430244326</v>
+        <v>-0.6701959009609251</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6640</v>
+        <v>6667</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>366.708003289398</v>
+        <v>363.4068678810371</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>995</v>
+        <v>255</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>38.78904336163709</v>
+        <v>40.36420614039848</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>19.61234233846608</v>
+        <v>11.25283339005108</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.6161250987838414</v>
+        <v>0.326947522433445</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>2.992810436708212</v>
+        <v>-2.09710506603584</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6588</v>
+        <v>6695</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>365.7707035167654</v>
+        <v>354.5040666521084</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>78.90000000000001</v>
+        <v>53.7</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>27.44225560475532</v>
+        <v>44.25081250665493</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.34932604040345</v>
+        <v>20.01410549803342</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.5217914986181071</v>
+        <v>0.2781308503205539</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.6701959009609251</v>
+        <v>-1.002137708427648</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6667</v>
+        <v>6768</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>363.4068678810371</v>
+        <v>351.2708120455608</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>255</v>
+        <v>71.2</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>40.36420614039848</v>
+        <v>26.43697351487201</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.25283339005108</v>
+        <v>28.28702706409566</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.326947522433445</v>
+        <v>0.5996688685354499</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-2.09710506603584</v>
+        <v>-1.143813432097494</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6695</v>
+        <v>6689</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>354.5040666521084</v>
+        <v>344.0970528510371</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>53.7</v>
+        <v>63.8</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>44.25081250665493</v>
+        <v>41.37266848906904</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>20.01410549803342</v>
+        <v>15.33572375315994</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.2781308503205539</v>
+        <v>0.3667007007287019</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-1.002137708427648</v>
+        <v>-0.0371268968194189</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6768</v>
+        <v>6531</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>351.2708120455608</v>
+        <v>343.755448438344</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>71.2</v>
+        <v>922</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>26.43697351487201</v>
+        <v>44.93989250651241</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>28.28702706409566</v>
+        <v>19.70161541490256</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.5996688685354499</v>
+        <v>0.6913528299949102</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-1.143813432097494</v>
+        <v>-13.47024695107131</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6689</v>
+        <v>6584</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>344.0970528510371</v>
+        <v>341.5014138720194</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>63.8</v>
+        <v>663</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.37266848906904</v>
+        <v>48.49963351571066</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>15.33572375315994</v>
+        <v>13.68941483089875</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.3667007007287019</v>
+        <v>0.250640185268231</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0371268968194189</v>
+        <v>-1.546796010479504</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6584</v>
+        <v>6515</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>341.5014138720194</v>
+        <v>336.1627714219665</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>663</v>
+        <v>7765</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,29 +5746,29 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>48.49963351571066</v>
+        <v>40.32504192944973</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>13.68941483089875</v>
+        <v>15.73228471199892</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.250640185268231</v>
+        <v>0.7537787896570529</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M100" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-1.546796010479504</v>
+        <v>-129.3450513143999</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, dealer_buy_3d</t>
         </is>
       </c>
     </row>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6533</v>
+        <v>6761</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>271.019284031169</v>
+        <v>265.8147523292832</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>191.5</v>
+        <v>181</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>39.34478541705536</v>
+        <v>42.60938299468615</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>9.453825813729642</v>
+        <v>12.64427604056821</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4116433795171787</v>
+        <v>0.9961010342967304</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.06783734416913841</v>
+        <v>-0.9036602854693992</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6761</v>
+        <v>6498</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>265.8147523292832</v>
+        <v>261.1769073280221</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>181</v>
+        <v>91.8</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>42.60938299468615</v>
+        <v>41.4882705419237</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>12.64427604056821</v>
+        <v>18.97596249194498</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.9961010342967304</v>
+        <v>0.3255869692953529</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.9036602854693992</v>
+        <v>-0.9173587365460693</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6498</v>
+        <v>6605</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>261.1769073280221</v>
+        <v>255.499487966438</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>91.8</v>
+        <v>126</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>41.4882705419237</v>
+        <v>33.57567588141866</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.97596249194498</v>
+        <v>13.53493576345398</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3255869692953529</v>
+        <v>2.449948796643803</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>1</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.9173587365460693</v>
+        <v>-1.289102728643541</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6605</v>
+        <v>6533</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>255.499487966438</v>
+        <v>251.019284031169</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>126</v>
+        <v>191.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>33.57567588141866</v>
+        <v>39.34478541705536</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>13.53493576345398</v>
+        <v>9.453825813729642</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>2.449948796643803</v>
+        <v>0.4116433795171787</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-1.289102728643541</v>
+        <v>0.06783734416913841</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6643</v>
+        <v>6558</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>246.7443182003722</v>
+        <v>248.1066860659051</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>442</v>
+        <v>29.8</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>35.73910293436239</v>
+        <v>46.94589364220873</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>18.79145957529873</v>
+        <v>16.41761503232766</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.104121604883709</v>
+        <v>0.4195210839764871</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1686557511894655</v>
+        <v>0.0660881360678495</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6692</v>
+        <v>6674</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>246.6309442467248</v>
+        <v>247.3706975194452</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>25</v>
+        <v>16.8</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>41.72174719942128</v>
+        <v>40.38139183846709</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>12.54193452547294</v>
+        <v>18.13934322261268</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.2419352251399605</v>
+        <v>0.4983078002169389</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0209835230382586</v>
+        <v>-0.0226857405212607</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6622,21 +6622,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6803</v>
+        <v>6643</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>239.9642073391053</v>
+        <v>246.7443182003722</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>274</v>
+        <v>442</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>28.53793049864439</v>
+        <v>35.73910293436239</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>36.65968903144845</v>
+        <v>18.79145957529873</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.2369421464651919</v>
+        <v>1.104121604883709</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-1.579237518361683</v>
+        <v>-0.1686557511894655</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6532</v>
+        <v>6692</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>進能服</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>237.9545737167573</v>
+        <v>246.6309442467248</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>31.24913595285118</v>
+        <v>41.72174719942128</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>16.1545400091649</v>
+        <v>12.54193452547294</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.7762651967701159</v>
+        <v>0.2419352251399605</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.9832574008631489</v>
+        <v>0.0209835230382586</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6807</v>
+        <v>6803</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>224.0150085429477</v>
+        <v>239.9642073391053</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>33.35</v>
+        <v>274</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>46.52416976153248</v>
+        <v>28.53793049864439</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>13.95221314332964</v>
+        <v>36.65968903144845</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.333634743756815</v>
+        <v>0.2369421464651919</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.07533203571149159</v>
+        <v>-1.579237518361683</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6546</v>
+        <v>6532</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>223.4927247787704</v>
+        <v>237.9545737167573</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>67.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>40.83189033534597</v>
+        <v>31.24913595285118</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>13.29868819812367</v>
+        <v>16.1545400091649</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.752247196514949</v>
+        <v>0.7762651967701159</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>1</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.3719280812801768</v>
+        <v>-0.9832574008631489</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6558</v>
+        <v>6591</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>218.1066860659051</v>
+        <v>231.8795914127692</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>29.8</v>
+        <v>49.4</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>46.94589364220873</v>
+        <v>31.54900827599663</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>16.41761503232766</v>
+        <v>22.90409423219014</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.4195210839764871</v>
+        <v>1.305711264294257</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0660881360678495</v>
+        <v>-0.4216307764317983</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6674</v>
+        <v>6807</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>217.3706975194452</v>
+        <v>224.0150085429477</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>16.8</v>
+        <v>33.35</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>40.38139183846709</v>
+        <v>46.52416976153248</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.13934322261268</v>
+        <v>13.95221314332964</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.4983078002169389</v>
+        <v>0.333634743756815</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0226857405212607</v>
+        <v>0.07533203571149159</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6680</v>
+        <v>6546</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>鑫創電子</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>215.1806078656739</v>
+        <v>223.4927247787704</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>49.35</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>50.04762709247905</v>
+        <v>40.83189033534597</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>3.979599990881894</v>
+        <v>13.29868819812367</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.0916956364419161</v>
+        <v>0.752247196514949</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0930235033627497</v>
+        <v>-0.3719280812801768</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6706</v>
+        <v>6680</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>鑫創電子</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>211.513259131728</v>
+        <v>215.1806078656739</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>139</v>
+        <v>49.35</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.54028330554185</v>
+        <v>50.04762709247905</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>16.35562291396795</v>
+        <v>3.979599990881894</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.2773792467241036</v>
+        <v>0.0916956364419161</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-1.519361429137161</v>
+        <v>0.0930235033627497</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6591</v>
+        <v>6706</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>201.8795914127692</v>
+        <v>211.513259131728</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>49.4</v>
+        <v>139</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>31.54900827599663</v>
+        <v>37.54028330554185</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>22.90409423219014</v>
+        <v>16.35562291396795</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>1.305711264294257</v>
+        <v>0.2773792467241036</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.4216307764317983</v>
+        <v>-1.519361429137161</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6754</v>
+        <v>6552</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>179.8881303456991</v>
+        <v>180.7910911011637</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>41.5</v>
+        <v>29.45</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,16 +7124,16 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>31.97657396369875</v>
+        <v>45.23529014758144</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>18.93448359424568</v>
+        <v>11.04092161165751</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.5416796400835713</v>
+        <v>0.6252321844502756</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L126" s="2" t="n">
         <v>0</v>
@@ -7142,31 +7142,31 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.398411468954379</v>
+        <v>-0.08376396779094911</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>6552</v>
+        <v>6754</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>150.7910911011637</v>
+        <v>179.8881303456991</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>29.45</v>
+        <v>41.5</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,16 +7177,16 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>45.23529014758144</v>
+        <v>31.97657396369875</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>11.04092161165751</v>
+        <v>18.93448359424568</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.6252321844502756</v>
+        <v>0.5416796400835713</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L127" s="2" t="n">
         <v>0</v>
@@ -7195,11 +7195,11 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.08376396779094911</v>
+        <v>-0.398411468954379</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scan: seg6 2026-07-10 20:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-09.xlsx
@@ -898,21 +898,21 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6782</v>
+        <v>6579</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>視陽</t>
+          <t>研揚</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>816.4694015700398</v>
+        <v>830.0519318813801</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,16 +923,16 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>61.2161079898446</v>
+        <v>55.65079568800395</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>18.98883101348961</v>
+        <v>22.69065329718225</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.738489463039223</v>
+        <v>0.92462148803372</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.851998813488339</v>
+        <v>0.7628516712453965</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6790</v>
+        <v>6782</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>永豐實</t>
+          <t>視陽</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>797.5848642475654</v>
+        <v>816.4694015700398</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>40.6</v>
+        <v>208</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,16 +976,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>56.06017041130701</v>
+        <v>61.2161079898446</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>27.42534162084732</v>
+        <v>18.98883101348961</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>2.216894408836775</v>
+        <v>1.738489463039223</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0200650518973029</v>
+        <v>1.851998813488339</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6579</v>
+        <v>6672</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>研揚</t>
+          <t>騰輝電子-KY</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>790.0519318813801</v>
+        <v>813.9820381707417</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>168</v>
+        <v>298</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>55.65079568800395</v>
+        <v>63.28453907555873</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>22.69065329718225</v>
+        <v>44.90669516572874</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.92462148803372</v>
+        <v>0.4074601068240206</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.7628516712453965</v>
+        <v>0.909622065573938</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1057,21 +1057,21 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6672</v>
+        <v>6790</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>騰輝電子-KY</t>
+          <t>永豐實</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>773.9820381707417</v>
+        <v>797.5848642475654</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>298</v>
+        <v>40.6</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63.28453907555873</v>
+        <v>56.06017041130701</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>44.90669516572874</v>
+        <v>27.42534162084732</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.4074601068240206</v>
+        <v>2.216894408836775</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,11 +1100,11 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.909622065573938</v>
+        <v>0.0200650518973029</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>745.1053716558544</v>
+        <v>785.1053716558544</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>199.5</v>
@@ -1852,21 +1852,21 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6494</v>
+        <v>6526</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>605.6281069906465</v>
+        <v>620.8358868881099</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>65.40000000000001</v>
+        <v>652</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,49 +1877,49 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>54.75708981889597</v>
+        <v>46.55920794044477</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>30.79711053846729</v>
+        <v>12.50977640156015</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.4960974403011379</v>
+        <v>0.3180578006867144</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.4436447065226803</v>
+        <v>-3.836454092270575</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6548</v>
+        <v>6494</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>長科*</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>605.0684096141974</v>
+        <v>605.6281069906465</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>82.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,49 +1930,49 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>49.32164392833502</v>
+        <v>54.75708981889597</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>35.19220546615367</v>
+        <v>30.79711053846729</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.4280797026316167</v>
+        <v>0.4960974403011379</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-1.606830051550298</v>
+        <v>-0.4436447065226803</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6776</v>
+        <v>6548</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>長科*</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>602.1172151615042</v>
+        <v>605.0684096141974</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>55.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,49 +1983,49 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>44.07719400615863</v>
+        <v>49.32164392833502</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>15.16728503789413</v>
+        <v>35.19220546615367</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.4556270969896387</v>
+        <v>0.4280797026316167</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M29" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.007830528605297499</v>
+        <v>-1.606830051550298</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6719</v>
+        <v>6776</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>力智</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>600.4071475628472</v>
+        <v>602.1172151615042</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>266.5</v>
+        <v>55.7</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.77748288044828</v>
+        <v>44.07719400615863</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>36.36714290865228</v>
+        <v>15.16728503789413</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.4679120686323972</v>
+        <v>0.4556270969896387</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-2.178105202121177</v>
+        <v>0.007830528605297499</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6534</v>
+        <v>6719</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>正瀚-創</t>
+          <t>力智</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>596.5304830346231</v>
+        <v>600.4071475628472</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>93</v>
+        <v>266.5</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>56.377685820084</v>
+        <v>50.77748288044828</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>15.95026664477515</v>
+        <v>36.36714290865228</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1.365323079628226</v>
+        <v>0.4679120686323972</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.3359677804920924</v>
+        <v>-2.178105202121177</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6651</v>
+        <v>6534</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>全宇昕</t>
+          <t>正瀚-創</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>596.327139434096</v>
+        <v>596.5304830346231</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>153</v>
+        <v>93</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>52.85462862539603</v>
+        <v>56.377685820084</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>29.15820876787029</v>
+        <v>15.95026664477515</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.5657071327213851</v>
+        <v>1.365323079628226</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.3302301955753322</v>
+        <v>0.3359677804920924</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6693</v>
+        <v>6651</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>廣閎科</t>
+          <t>全宇昕</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>592.7668022939393</v>
+        <v>596.327139434096</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>236.5</v>
+        <v>153</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>57.38882725730897</v>
+        <v>52.85462862539603</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>48.35219013904855</v>
+        <v>29.15820876787029</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.7093456386997857</v>
+        <v>0.5657071327213851</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.8913554387701943</v>
+        <v>-0.3302301955753322</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6829</v>
+        <v>6693</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>千附精密</t>
+          <t>廣閎科</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>582.0746388788924</v>
+        <v>592.7668022939393</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>222</v>
+        <v>236.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>53.37132264412852</v>
+        <v>57.38882725730897</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>12.80794466052242</v>
+        <v>48.35219013904855</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.029161936934242</v>
+        <v>0.7093456386997857</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.134213562158755</v>
+        <v>-0.8913554387701943</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6526</v>
+        <v>6829</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>千附精密</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>580.8358868881099</v>
+        <v>582.0746388788924</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>652</v>
+        <v>222</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,29 +2301,29 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>46.55920794044477</v>
+        <v>53.37132264412852</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>12.50977640156015</v>
+        <v>12.80794466052242</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.3180578006867144</v>
+        <v>1.029161936934242</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-3.836454092270575</v>
+        <v>0.134213562158755</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6757</v>
+        <v>6641</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>台灣虎航-創</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>539.6201191390852</v>
+        <v>541.3480499949726</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>58.2</v>
+        <v>18.55</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>47.89947150532576</v>
+        <v>52.15916601029208</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>33.4044542250839</v>
+        <v>21.53463700116355</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.3874529482200982</v>
+        <v>0.2348049994972524</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.510026576499796</v>
+        <v>0.0789543981768993</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6556</v>
+        <v>6757</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>台灣虎航-創</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>537.7912947879956</v>
+        <v>539.6201191390852</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>70.59999999999999</v>
+        <v>58.2</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>43.50049532804022</v>
+        <v>47.89947150532576</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>25.4175389739355</v>
+        <v>33.4044542250839</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>4.507926746338204</v>
+        <v>0.3874529482200982</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.193538167136914</v>
+        <v>-0.510026576499796</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6613</v>
+        <v>6556</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>朋億*</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>532.2781759184518</v>
+        <v>537.7912947879956</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>321</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>48.1548853306832</v>
+        <v>43.50049532804022</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>26.18091668333613</v>
+        <v>25.4175389739355</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.3491639708233205</v>
+        <v>4.507926746338204</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-8.294732397284093</v>
+        <v>-0.193538167136914</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6486</v>
+        <v>6668</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>互動</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>526.4315539908017</v>
+        <v>534.0954600328597</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>83.09999999999999</v>
+        <v>37.9</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>54.46584108495598</v>
+        <v>44.24061600837763</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>22.52926446869758</v>
+        <v>17.49634825636789</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.7014900816502103</v>
+        <v>0.2315904586944201</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.2434784200002912</v>
+        <v>-0.5166812948567168</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6541</v>
+        <v>6613</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>朋億*</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>520.788563706419</v>
+        <v>532.2781759184518</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>40.8</v>
+        <v>321</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>50.37825055393518</v>
+        <v>48.1548853306832</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>15.95431463490334</v>
+        <v>26.18091668333613</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.4791819830682827</v>
+        <v>0.3491639708233205</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.0515945649777843</v>
+        <v>-8.294732397284093</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6684</v>
+        <v>6669</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>安格</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>513.5871514814752</v>
+        <v>527.7527193266883</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>53.9</v>
+        <v>5040</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,49 +3043,49 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>48.12188760072574</v>
+        <v>51.96524510439431</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>34.74033046096234</v>
+        <v>13.16601854784374</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.2555517275361595</v>
+        <v>1.239935985599949</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.844057614690052</v>
+        <v>35.82695697358312</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6722</v>
+        <v>6486</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>509.7704691092051</v>
+        <v>526.4315539908017</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>35.45</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>41.78422157427065</v>
+        <v>54.46584108495598</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>36.62134005229357</v>
+        <v>22.52926446869758</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.1865728134092482</v>
+        <v>0.7014900816502103</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.0319693211539622</v>
+        <v>0.2434784200002912</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6771</v>
+        <v>6541</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>505.9485006770078</v>
+        <v>520.788563706419</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>39.8</v>
+        <v>40.8</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>44.11121485010584</v>
+        <v>50.37825055393518</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>20.97283053484768</v>
+        <v>15.95431463490334</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.3808665749470042</v>
+        <v>0.4791819830682827</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0462064449937836</v>
+        <v>-0.0515945649777843</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6641</v>
+        <v>6684</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>安格</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>501.3480499949725</v>
+        <v>513.5871514814752</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>18.55</v>
+        <v>53.9</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.15916601029208</v>
+        <v>48.12188760072574</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>21.53463700116355</v>
+        <v>34.74033046096234</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.2348049994972524</v>
+        <v>0.2555517275361595</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0789543981768993</v>
+        <v>-0.844057614690052</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6756</v>
+        <v>6722</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>498.5706487819775</v>
+        <v>509.7704691092051</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>99.7</v>
+        <v>35.45</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>51.11622393290391</v>
+        <v>41.78422157427065</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.43002931375125</v>
+        <v>36.62134005229357</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.719580924508797</v>
+        <v>0.1865728134092482</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.0941166256695159</v>
+        <v>0.0319693211539622</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6805</v>
+        <v>6771</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>498.2261690857841</v>
+        <v>505.9485006770078</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>1460</v>
+        <v>39.8</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>35.04999473985863</v>
+        <v>44.11121485010584</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>23.31580815943655</v>
+        <v>20.97283053484768</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.466381395435663</v>
+        <v>0.3808665749470042</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-27.45016259752049</v>
+        <v>0.0462064449937836</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6530</v>
+        <v>6756</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>496.8663280777081</v>
+        <v>498.5706487819775</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>83</v>
+        <v>99.7</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>35.42061692529114</v>
+        <v>51.11622393290391</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>22.55340177651775</v>
+        <v>18.43002931375125</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.6051592319693341</v>
+        <v>0.719580924508797</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.1612898038329095</v>
+        <v>-0.0941166256695159</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6668</v>
+        <v>6805</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>494.0954600328597</v>
+        <v>498.2261690857841</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>37.9</v>
+        <v>1460</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.24061600837763</v>
+        <v>35.04999473985863</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>17.49634825636789</v>
+        <v>23.31580815943655</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2315904586944201</v>
+        <v>1.466381395435663</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.5166812948567168</v>
+        <v>-27.45016259752049</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6669</v>
+        <v>6530</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>487.7527193266883</v>
+        <v>496.8663280777081</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>5040</v>
+        <v>83</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,29 +3467,29 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.96524510439431</v>
+        <v>35.42061692529114</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>13.16601854784374</v>
+        <v>22.55340177651775</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>1.239935985599949</v>
+        <v>0.6051592319693341</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>35.82695697358312</v>
+        <v>-0.1612898038329095</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -3548,21 +3548,21 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6691</v>
+        <v>6581</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>洋基工程</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>484.1849016766411</v>
+        <v>487.4493408512781</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>708</v>
+        <v>106.5</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>47.83081928113256</v>
+        <v>43.64214916955456</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>26.21879230494516</v>
+        <v>11.34799022438651</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.3184901676641075</v>
+        <v>1.861734772157725</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-8.401246741242378</v>
+        <v>-0.0759752293400259</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6830</v>
+        <v>6691</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>汎銓</t>
+          <t>洋基工程</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>482.9114658730273</v>
+        <v>484.1849016766411</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>416.5</v>
+        <v>708</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>31.57675210294522</v>
+        <v>47.83081928113256</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>25.83060349809814</v>
+        <v>26.21879230494516</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.8696450274370079</v>
+        <v>0.3184901676641075</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-4.110552602012078</v>
+        <v>-8.401246741242378</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6788</v>
+        <v>6830</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>汎銓</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>481.9701892520345</v>
+        <v>482.9114658730273</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>403.5</v>
+        <v>416.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,49 +3679,49 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>42.06927033991832</v>
+        <v>31.57675210294522</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>8.618651842756288</v>
+        <v>25.83060349809814</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4669477995439862</v>
+        <v>0.8696450274370079</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M61" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-3.771028098114664</v>
+        <v>-4.110552602012078</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6614</v>
+        <v>6788</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>472.1724104726767</v>
+        <v>481.9701892520345</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>40</v>
+        <v>403.5</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,49 +3732,49 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.11212072275216</v>
+        <v>42.06927033991832</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>20.77426729531906</v>
+        <v>8.618651842756288</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.4194081595047057</v>
+        <v>0.4669477995439862</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M62" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0148271299643166</v>
+        <v>-3.771028098114664</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6581</v>
+        <v>6614</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>467.4493408512781</v>
+        <v>472.1724104726767</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>106.5</v>
+        <v>40</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>43.64214916955456</v>
+        <v>49.11212072275216</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>11.34799022438651</v>
+        <v>20.77426729531906</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.861734772157725</v>
+        <v>0.4194081595047057</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>1</v>
@@ -3803,11 +3803,11 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.0759752293400259</v>
+        <v>0.0148271299643166</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6725</v>
+        <v>6531</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>383.5367904348528</v>
+        <v>383.7554484383441</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>305.5</v>
+        <v>922</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.21693973076976</v>
+        <v>44.93989250651241</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>21.50047520525937</v>
+        <v>19.70161541490256</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.1970419132930303</v>
+        <v>0.6913528299949102</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-3.411320418058653</v>
+        <v>-13.47024695107131</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6561</v>
+        <v>6725</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>381.3219879093637</v>
+        <v>383.5367904348528</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>330.5</v>
+        <v>305.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>39.09196338881269</v>
+        <v>43.21693973076976</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>20.63001740319667</v>
+        <v>21.50047520525937</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.3129231034568797</v>
+        <v>0.1970419132930303</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.1680527533914375</v>
+        <v>-3.411320418058653</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6690</v>
+        <v>6561</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>379.4332732063193</v>
+        <v>381.3219879093637</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>166.5</v>
+        <v>330.5</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,16 +4951,16 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>44.63014541075785</v>
+        <v>39.09196338881269</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>14.43662579867491</v>
+        <v>20.63001740319667</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.3219020244547579</v>
+        <v>0.3129231034568797</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.3006336229487034</v>
+        <v>-0.1680527533914375</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6789</v>
+        <v>6690</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>采鈺</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>378.5211467168094</v>
+        <v>379.4332732063193</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>515</v>
+        <v>166.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>49.29976006274612</v>
+        <v>44.63014541075785</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>11.45613657085052</v>
+        <v>14.43662579867491</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.5078244177819691</v>
+        <v>0.3219020244547579</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>4</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.7010781471795562</v>
+        <v>-0.3006336229487034</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6597</v>
+        <v>6789</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>采鈺</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>376.4787716480552</v>
+        <v>378.5211467168094</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>67.8</v>
+        <v>515</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>51.52220358926256</v>
+        <v>49.29976006274612</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>14.4416454967116</v>
+        <v>11.45613657085052</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.2217467632214176</v>
+        <v>0.5078244177819691</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-2.553841087692786</v>
+        <v>-0.7010781471795562</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, williams_r_recovery</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6715</v>
+        <v>6597</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>375.7961387345421</v>
+        <v>376.4787716480552</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>391.5</v>
+        <v>67.8</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>41.02153305558943</v>
+        <v>51.52220358926256</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>17.16508098089622</v>
+        <v>14.4416454967116</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>2.332115911198549</v>
+        <v>0.2217467632214176</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-6.670494945067979</v>
+        <v>-2.553841087692786</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6741</v>
+        <v>6515</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>375.1821582725876</v>
+        <v>376.1627714219665</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>60</v>
+        <v>7765</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,49 +5163,49 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>40.98150273237917</v>
+        <v>40.32504192944973</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>9.099618418777792</v>
+        <v>15.73228471199892</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>1.474235345176557</v>
+        <v>0.7537787896570529</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M89" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.1252753070053037</v>
+        <v>-129.3450513143999</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6510</v>
+        <v>6715</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>372.8793682236349</v>
+        <v>375.7961387345421</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>2855</v>
+        <v>391.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,49 +5216,49 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>37.5037168934422</v>
+        <v>41.02153305558943</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>20.50776648792229</v>
+        <v>17.16508098089622</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.6169599725795567</v>
+        <v>2.332115911198549</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M90" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-53.90204377594968</v>
+        <v>-6.670494945067979</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6763</v>
+        <v>6741</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>372.2888543904213</v>
+        <v>375.1821582725876</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>45.9</v>
+        <v>60</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>44.24551976832949</v>
+        <v>40.98150273237917</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>14.3906360408211</v>
+        <v>9.099618418777792</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.7669989018105312</v>
+        <v>1.474235345176557</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1506834430244326</v>
+        <v>-0.1252753070053037</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6640</v>
+        <v>6510</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>366.708003289398</v>
+        <v>372.8793682236349</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>995</v>
+        <v>2855</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,49 +5322,49 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>38.78904336163709</v>
+        <v>37.5037168934422</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>19.61234233846608</v>
+        <v>20.50776648792229</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.6161250987838414</v>
+        <v>0.6169599725795567</v>
       </c>
       <c r="K92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L92" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M92" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>2.992810436708212</v>
+        <v>-53.90204377594968</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6588</v>
+        <v>6763</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>365.7707035167654</v>
+        <v>372.2888543904213</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>78.90000000000001</v>
+        <v>45.9</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>27.44225560475532</v>
+        <v>44.24551976832949</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>21.34932604040345</v>
+        <v>14.3906360408211</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5217914986181071</v>
+        <v>0.7669989018105312</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.6701959009609251</v>
+        <v>-0.1506834430244326</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6667</v>
+        <v>6640</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>363.4068678810371</v>
+        <v>366.708003289398</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>255</v>
+        <v>995</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.36420614039848</v>
+        <v>38.78904336163709</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>11.25283339005108</v>
+        <v>19.61234233846608</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.326947522433445</v>
+        <v>0.6161250987838414</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-2.09710506603584</v>
+        <v>2.992810436708212</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6695</v>
+        <v>6588</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>354.5040666521084</v>
+        <v>365.7707035167654</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>53.7</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.25081250665493</v>
+        <v>27.44225560475532</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>20.01410549803342</v>
+        <v>21.34932604040345</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.2781308503205539</v>
+        <v>0.5217914986181071</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.002137708427648</v>
+        <v>-0.6701959009609251</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6768</v>
+        <v>6667</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>351.2708120455608</v>
+        <v>363.4068678810371</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>71.2</v>
+        <v>255</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>26.43697351487201</v>
+        <v>40.36420614039848</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>28.28702706409566</v>
+        <v>11.25283339005108</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.5996688685354499</v>
+        <v>0.326947522433445</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-1.143813432097494</v>
+        <v>-2.09710506603584</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6689</v>
+        <v>6695</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>344.0970528510371</v>
+        <v>354.5040666521084</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>63.8</v>
+        <v>53.7</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>41.37266848906904</v>
+        <v>44.25081250665493</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>15.33572375315994</v>
+        <v>20.01410549803342</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3667007007287019</v>
+        <v>0.2781308503205539</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.0371268968194189</v>
+        <v>-1.002137708427648</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6531</v>
+        <v>6768</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>343.755448438344</v>
+        <v>351.2708120455608</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>922</v>
+        <v>71.2</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>44.93989250651241</v>
+        <v>26.43697351487201</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.70161541490256</v>
+        <v>28.28702706409566</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.6913528299949102</v>
+        <v>0.5996688685354499</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-13.47024695107131</v>
+        <v>-1.143813432097494</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6584</v>
+        <v>6689</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>341.5014138720194</v>
+        <v>344.0970528510371</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>663</v>
+        <v>63.8</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>48.49963351571066</v>
+        <v>41.37266848906904</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>13.68941483089875</v>
+        <v>15.33572375315994</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.250640185268231</v>
+        <v>0.3667007007287019</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-1.546796010479504</v>
+        <v>-0.0371268968194189</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6515</v>
+        <v>6584</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>336.1627714219665</v>
+        <v>341.5014138720194</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>7765</v>
+        <v>663</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,29 +5746,29 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>40.32504192944973</v>
+        <v>48.49963351571066</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>15.73228471199892</v>
+        <v>13.68941483089875</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.7537787896570529</v>
+        <v>0.250640185268231</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M100" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-129.3450513143999</v>
+        <v>-1.546796010479504</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6761</v>
+        <v>6533</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>265.8147523292832</v>
+        <v>271.019284031169</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>181</v>
+        <v>191.5</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.60938299468615</v>
+        <v>39.34478541705536</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>12.64427604056821</v>
+        <v>9.453825813729642</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.9961010342967304</v>
+        <v>0.4116433795171787</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.9036602854693992</v>
+        <v>0.06783734416913841</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6498</v>
+        <v>6761</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>261.1769073280221</v>
+        <v>265.8147523292832</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>91.8</v>
+        <v>181</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>41.4882705419237</v>
+        <v>42.60938299468615</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>18.97596249194498</v>
+        <v>12.64427604056821</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.3255869692953529</v>
+        <v>0.9961010342967304</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.9173587365460693</v>
+        <v>-0.9036602854693992</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6605</v>
+        <v>6498</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>255.499487966438</v>
+        <v>261.1769073280221</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>126</v>
+        <v>91.8</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>33.57567588141866</v>
+        <v>41.4882705419237</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>13.53493576345398</v>
+        <v>18.97596249194498</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>2.449948796643803</v>
+        <v>0.3255869692953529</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>1</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-1.289102728643541</v>
+        <v>-0.9173587365460693</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6533</v>
+        <v>6605</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>251.019284031169</v>
+        <v>255.499487966438</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>191.5</v>
+        <v>126</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>39.34478541705536</v>
+        <v>33.57567588141866</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>9.453825813729642</v>
+        <v>13.53493576345398</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.4116433795171787</v>
+        <v>2.449948796643803</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.06783734416913841</v>
+        <v>-1.289102728643541</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6558</v>
+        <v>6643</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>248.1066860659051</v>
+        <v>246.7443182003722</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>29.8</v>
+        <v>442</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>46.94589364220873</v>
+        <v>35.73910293436239</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>16.41761503232766</v>
+        <v>18.79145957529873</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.4195210839764871</v>
+        <v>1.104121604883709</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0660881360678495</v>
+        <v>-0.1686557511894655</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6674</v>
+        <v>6692</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>進能服</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>247.3706975194452</v>
+        <v>246.6309442467248</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>16.8</v>
+        <v>25</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>40.38139183846709</v>
+        <v>41.72174719942128</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>18.13934322261268</v>
+        <v>12.54193452547294</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.4983078002169389</v>
+        <v>0.2419352251399605</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.0226857405212607</v>
+        <v>0.0209835230382586</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6622,21 +6622,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6643</v>
+        <v>6803</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>246.7443182003722</v>
+        <v>239.9642073391053</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>442</v>
+        <v>274</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>35.73910293436239</v>
+        <v>28.53793049864439</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>18.79145957529873</v>
+        <v>36.65968903144845</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>1.104121604883709</v>
+        <v>0.2369421464651919</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1686557511894655</v>
+        <v>-1.579237518361683</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6692</v>
+        <v>6532</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>瑞耘</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>246.6309442467248</v>
+        <v>237.9545737167573</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>41.72174719942128</v>
+        <v>31.24913595285118</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>12.54193452547294</v>
+        <v>16.1545400091649</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.2419352251399605</v>
+        <v>0.7762651967701159</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0209835230382586</v>
+        <v>-0.9832574008631489</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6803</v>
+        <v>6807</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>239.9642073391053</v>
+        <v>224.0150085429477</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>274</v>
+        <v>33.35</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>28.53793049864439</v>
+        <v>46.52416976153248</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>36.65968903144845</v>
+        <v>13.95221314332964</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.2369421464651919</v>
+        <v>0.333634743756815</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-1.579237518361683</v>
+        <v>0.07533203571149159</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6532</v>
+        <v>6546</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>瑞耘</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>237.9545737167573</v>
+        <v>223.4927247787704</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>78</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>31.24913595285118</v>
+        <v>40.83189033534597</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>16.1545400091649</v>
+        <v>13.29868819812367</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.7762651967701159</v>
+        <v>0.752247196514949</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>1</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.9832574008631489</v>
+        <v>-0.3719280812801768</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6591</v>
+        <v>6558</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>231.8795914127692</v>
+        <v>218.1066860659051</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>49.4</v>
+        <v>29.8</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>31.54900827599663</v>
+        <v>46.94589364220873</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>22.90409423219014</v>
+        <v>16.41761503232766</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.305711264294257</v>
+        <v>0.4195210839764871</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.4216307764317983</v>
+        <v>0.0660881360678495</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6807</v>
+        <v>6674</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>224.0150085429477</v>
+        <v>217.3706975194452</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>33.35</v>
+        <v>16.8</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.52416976153248</v>
+        <v>40.38139183846709</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>13.95221314332964</v>
+        <v>18.13934322261268</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.333634743756815</v>
+        <v>0.4983078002169389</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.07533203571149159</v>
+        <v>-0.0226857405212607</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6546</v>
+        <v>6680</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>鑫創電子</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>223.4927247787704</v>
+        <v>215.1806078656739</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>67.59999999999999</v>
+        <v>49.35</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>40.83189033534597</v>
+        <v>50.04762709247905</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.29868819812367</v>
+        <v>3.979599990881894</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.752247196514949</v>
+        <v>0.0916956364419161</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.3719280812801768</v>
+        <v>0.0930235033627497</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6680</v>
+        <v>6706</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>鑫創電子</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>215.1806078656739</v>
+        <v>211.513259131728</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>49.35</v>
+        <v>139</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>50.04762709247905</v>
+        <v>37.54028330554185</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>3.979599990881894</v>
+        <v>16.35562291396795</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.0916956364419161</v>
+        <v>0.2773792467241036</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0930235033627497</v>
+        <v>-1.519361429137161</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6706</v>
+        <v>6591</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>211.513259131728</v>
+        <v>201.8795914127692</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>139</v>
+        <v>49.4</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>37.54028330554185</v>
+        <v>31.54900827599663</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.35562291396795</v>
+        <v>22.90409423219014</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.2773792467241036</v>
+        <v>1.305711264294257</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.519361429137161</v>
+        <v>-0.4216307764317983</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6552</v>
+        <v>6754</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>180.7910911011637</v>
+        <v>179.8881303456991</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>29.45</v>
+        <v>41.5</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,16 +7124,16 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>45.23529014758144</v>
+        <v>31.97657396369875</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>11.04092161165751</v>
+        <v>18.93448359424568</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.6252321844502756</v>
+        <v>0.5416796400835713</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L126" s="2" t="n">
         <v>0</v>
@@ -7142,31 +7142,31 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.08376396779094911</v>
+        <v>-0.398411468954379</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>6754</v>
+        <v>6552</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>179.8881303456991</v>
+        <v>150.7910911011637</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>41.5</v>
+        <v>29.45</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,16 +7177,16 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>31.97657396369875</v>
+        <v>45.23529014758144</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>18.93448359424568</v>
+        <v>11.04092161165751</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.5416796400835713</v>
+        <v>0.6252321844502756</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L127" s="2" t="n">
         <v>0</v>
@@ -7195,11 +7195,11 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.398411468954379</v>
+        <v>-0.08376396779094911</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>

</xml_diff>